<commit_message>
Enhance Tender PO Invoice Edit and Quotation Edit Pages
- Updated the layout and styling of the Tender PO Invoice Edit page to improve user experience, including the addition of total amount calculations for additional charges.
- Implemented new sections for displaying total amounts excluding and including additional charges.
- Added functionality to dynamically load and display additional charges in the Tender PO Invoice Edit page.
- Modified the Tender Quotation Edit page to include serial numbers for items and improved the overall layout.
- Adjusted the Tender Quotation Print view to accommodate changes in column spans and added serial number display in the items table.
- Updated the sample Excel file for tender enquiry items to reflect recent changes.
</commit_message>
<xml_diff>
--- a/asset/tender-enquiry-items-sample.xlsx
+++ b/asset/tender-enquiry-items-sample.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Xampp\htdocs\erp-psm\asset\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>item_desc</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t>item_code</t>
+  </si>
+  <si>
+    <t>serial_no</t>
   </si>
 </sst>
 </file>
@@ -371,74 +374,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.26953125" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="1"/>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B17" s="1"/>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C16" s="1"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>